<commit_message>
fix: file uploads directApi + CargasModal import + ErrorBoundary
</commit_message>
<xml_diff>
--- a/scripts/nomina_prueba.xlsx
+++ b/scripts/nomina_prueba.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Nomina" sheetId="1" r:id="rId1"/>
+    <sheet name="Nómina Septiembre 2026" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -397,7 +397,24 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N12"/>
+  <dimension ref="A1:N13"/>
+  <cols>
+    <col min="1" max="1" width="16.83203125" customWidth="1"/>
+    <col min="2" max="2" width="12.83203125" customWidth="1"/>
+    <col min="3" max="3" width="14.83203125" customWidth="1"/>
+    <col min="4" max="4" width="12.83203125" customWidth="1"/>
+    <col min="5" max="5" width="18.83203125" customWidth="1"/>
+    <col min="6" max="6" width="14.83203125" customWidth="1"/>
+    <col min="7" max="7" width="15.83203125" customWidth="1"/>
+    <col min="8" max="8" width="20.83203125" customWidth="1"/>
+    <col min="9" max="9" width="14.83203125" customWidth="1"/>
+    <col min="10" max="10" width="14.83203125" customWidth="1"/>
+    <col min="11" max="11" width="12.83203125" customWidth="1"/>
+    <col min="12" max="12" width="16.83203125" customWidth="1"/>
+    <col min="13" max="13" width="16.83203125" customWidth="1"/>
+    <col min="14" max="14" width="14.83203125" customWidth="1"/>
+    <col min="15" max="15" width="14.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -445,43 +462,43 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>V-20.123.456</v>
+        <v>V-22.456.789</v>
       </c>
       <c r="B2">
-        <v>2800</v>
+        <v>3500</v>
       </c>
       <c r="C2">
-        <v>420</v>
+        <v>350</v>
       </c>
       <c r="D2">
-        <v>149.73</v>
+        <v>200</v>
       </c>
       <c r="E2">
-        <v>0</v>
+        <v>175</v>
       </c>
       <c r="F2">
-        <v>196.95</v>
+        <v>100</v>
       </c>
       <c r="G2">
-        <v>127.91</v>
+        <v>0</v>
       </c>
       <c r="H2">
-        <v>112</v>
+        <v>385</v>
       </c>
       <c r="I2">
-        <v>14</v>
+        <v>52.5</v>
       </c>
       <c r="J2">
-        <v>14</v>
+        <v>17.5</v>
       </c>
       <c r="K2">
-        <v>84</v>
+        <v>0</v>
       </c>
       <c r="L2">
-        <v>45</v>
+        <v>140</v>
       </c>
       <c r="M2">
-        <v>93.96</v>
+        <v>0</v>
       </c>
       <c r="N2">
         <v>0</v>
@@ -489,43 +506,43 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>V-25.987.654</v>
+        <v>V-20.123.456</v>
       </c>
       <c r="B3">
-        <v>2400</v>
+        <v>4500</v>
       </c>
       <c r="C3">
-        <v>360</v>
+        <v>450</v>
       </c>
       <c r="D3">
-        <v>208.05</v>
+        <v>300</v>
       </c>
       <c r="E3">
-        <v>0</v>
+        <v>225</v>
       </c>
       <c r="F3">
-        <v>165.64</v>
+        <v>150</v>
       </c>
       <c r="G3">
-        <v>94.09</v>
+        <v>200</v>
       </c>
       <c r="H3">
-        <v>96</v>
+        <v>495</v>
       </c>
       <c r="I3">
-        <v>12</v>
+        <v>67.5</v>
       </c>
       <c r="J3">
-        <v>12</v>
+        <v>22.5</v>
       </c>
       <c r="K3">
-        <v>72</v>
+        <v>150</v>
       </c>
       <c r="L3">
-        <v>45</v>
+        <v>180</v>
       </c>
       <c r="M3">
-        <v>6.34</v>
+        <v>0</v>
       </c>
       <c r="N3">
         <v>0</v>
@@ -533,43 +550,43 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>V-22.456.789</v>
+        <v>V-29.777.888</v>
       </c>
       <c r="B4">
-        <v>2200</v>
+        <v>2800</v>
       </c>
       <c r="C4">
-        <v>330</v>
+        <v>280</v>
       </c>
       <c r="D4">
-        <v>51.41</v>
+        <v>150</v>
       </c>
       <c r="E4">
-        <v>0</v>
+        <v>140</v>
       </c>
       <c r="F4">
-        <v>10</v>
+        <v>80</v>
       </c>
       <c r="G4">
-        <v>99.9</v>
+        <v>0</v>
       </c>
       <c r="H4">
-        <v>88</v>
+        <v>308</v>
       </c>
       <c r="I4">
-        <v>11</v>
+        <v>42</v>
       </c>
       <c r="J4">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="K4">
-        <v>66</v>
+        <v>0</v>
       </c>
       <c r="L4">
-        <v>45</v>
+        <v>112</v>
       </c>
       <c r="M4">
-        <v>153.23</v>
+        <v>0</v>
       </c>
       <c r="N4">
         <v>0</v>
@@ -577,43 +594,43 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>V-28.345.678</v>
+        <v>V-31.555.666</v>
       </c>
       <c r="B5">
-        <v>2600</v>
+        <v>3400</v>
       </c>
       <c r="C5">
-        <v>390</v>
+        <v>340</v>
       </c>
       <c r="D5">
-        <v>135.82</v>
+        <v>200</v>
       </c>
       <c r="E5">
-        <v>0</v>
+        <v>170</v>
       </c>
       <c r="F5">
-        <v>249.48</v>
+        <v>100</v>
       </c>
       <c r="G5">
-        <v>9.86</v>
+        <v>0</v>
       </c>
       <c r="H5">
-        <v>104</v>
+        <v>374</v>
       </c>
       <c r="I5">
-        <v>13</v>
+        <v>51</v>
       </c>
       <c r="J5">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="K5">
-        <v>78</v>
+        <v>0</v>
       </c>
       <c r="L5">
-        <v>45</v>
+        <v>136</v>
       </c>
       <c r="M5">
-        <v>127.06</v>
+        <v>0</v>
       </c>
       <c r="N5">
         <v>0</v>
@@ -621,43 +638,43 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>V-30.111.222</v>
+        <v>V-26.121.321</v>
       </c>
       <c r="B6">
-        <v>3200</v>
+        <v>2700</v>
       </c>
       <c r="C6">
-        <v>480</v>
+        <v>270</v>
       </c>
       <c r="D6">
-        <v>235.78</v>
+        <v>150</v>
       </c>
       <c r="E6">
-        <v>0</v>
+        <v>135</v>
       </c>
       <c r="F6">
-        <v>57.05</v>
+        <v>80</v>
       </c>
       <c r="G6">
-        <v>120.26</v>
+        <v>0</v>
       </c>
       <c r="H6">
-        <v>128</v>
+        <v>297</v>
       </c>
       <c r="I6">
-        <v>16</v>
+        <v>40.5</v>
       </c>
       <c r="J6">
-        <v>16</v>
+        <v>13.5</v>
       </c>
       <c r="K6">
-        <v>96</v>
+        <v>0</v>
       </c>
       <c r="L6">
-        <v>45</v>
+        <v>108</v>
       </c>
       <c r="M6">
-        <v>74.36</v>
+        <v>0</v>
       </c>
       <c r="N6">
         <v>0</v>
@@ -665,43 +682,43 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>V-31.555.666</v>
+        <v>V-30.111.222</v>
       </c>
       <c r="B7">
-        <v>2100</v>
+        <v>3200</v>
       </c>
       <c r="C7">
-        <v>315</v>
+        <v>320</v>
       </c>
       <c r="D7">
-        <v>196.42</v>
+        <v>200</v>
       </c>
       <c r="E7">
-        <v>0</v>
+        <v>160</v>
       </c>
       <c r="F7">
-        <v>107.96</v>
+        <v>100</v>
       </c>
       <c r="G7">
-        <v>127.66</v>
+        <v>150</v>
       </c>
       <c r="H7">
-        <v>84</v>
+        <v>352</v>
       </c>
       <c r="I7">
-        <v>10.5</v>
+        <v>48</v>
       </c>
       <c r="J7">
-        <v>10.5</v>
+        <v>16</v>
       </c>
       <c r="K7">
-        <v>63</v>
+        <v>100</v>
       </c>
       <c r="L7">
-        <v>45</v>
+        <v>128</v>
       </c>
       <c r="M7">
-        <v>131.01</v>
+        <v>0</v>
       </c>
       <c r="N7">
         <v>0</v>
@@ -709,43 +726,43 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>V-29.777.888</v>
+        <v>V-28.345.678</v>
       </c>
       <c r="B8">
-        <v>2500</v>
+        <v>3000</v>
       </c>
       <c r="C8">
-        <v>375</v>
+        <v>300</v>
       </c>
       <c r="D8">
-        <v>211.46</v>
+        <v>150</v>
       </c>
       <c r="E8">
-        <v>0</v>
+        <v>150</v>
       </c>
       <c r="F8">
-        <v>12.27</v>
+        <v>80</v>
       </c>
       <c r="G8">
-        <v>61.34</v>
+        <v>0</v>
       </c>
       <c r="H8">
-        <v>100</v>
+        <v>330</v>
       </c>
       <c r="I8">
-        <v>12.5</v>
+        <v>45</v>
       </c>
       <c r="J8">
-        <v>12.5</v>
+        <v>15</v>
       </c>
       <c r="K8">
-        <v>75</v>
+        <v>0</v>
       </c>
       <c r="L8">
-        <v>45</v>
+        <v>120</v>
       </c>
       <c r="M8">
-        <v>4.53</v>
+        <v>0</v>
       </c>
       <c r="N8">
         <v>0</v>
@@ -756,40 +773,40 @@
         <v>V-32.999.000</v>
       </c>
       <c r="B9">
-        <v>2300</v>
+        <v>2900</v>
       </c>
       <c r="C9">
-        <v>345</v>
+        <v>290</v>
       </c>
       <c r="D9">
-        <v>76.89</v>
+        <v>150</v>
       </c>
       <c r="E9">
-        <v>0</v>
+        <v>145</v>
       </c>
       <c r="F9">
-        <v>214.16</v>
+        <v>80</v>
       </c>
       <c r="G9">
-        <v>17.93</v>
+        <v>0</v>
       </c>
       <c r="H9">
-        <v>92</v>
+        <v>319</v>
       </c>
       <c r="I9">
-        <v>11.5</v>
+        <v>43.5</v>
       </c>
       <c r="J9">
-        <v>11.5</v>
+        <v>14.5</v>
       </c>
       <c r="K9">
-        <v>69</v>
+        <v>0</v>
       </c>
       <c r="L9">
-        <v>45</v>
+        <v>116</v>
       </c>
       <c r="M9">
-        <v>154.14</v>
+        <v>0</v>
       </c>
       <c r="N9">
         <v>0</v>
@@ -797,43 +814,43 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>V-26.121.321</v>
+        <v>V-25.987.654</v>
       </c>
       <c r="B10">
-        <v>2700</v>
+        <v>3800</v>
       </c>
       <c r="C10">
-        <v>405</v>
+        <v>380</v>
       </c>
       <c r="D10">
-        <v>219.37</v>
+        <v>250</v>
       </c>
       <c r="E10">
-        <v>0</v>
+        <v>190</v>
       </c>
       <c r="F10">
-        <v>123.03</v>
+        <v>120</v>
       </c>
       <c r="G10">
-        <v>101.36</v>
+        <v>100</v>
       </c>
       <c r="H10">
-        <v>108</v>
+        <v>418</v>
       </c>
       <c r="I10">
-        <v>13.5</v>
+        <v>57</v>
       </c>
       <c r="J10">
-        <v>13.5</v>
+        <v>19</v>
       </c>
       <c r="K10">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="L10">
-        <v>45</v>
+        <v>152</v>
       </c>
       <c r="M10">
-        <v>48.11</v>
+        <v>0</v>
       </c>
       <c r="N10">
         <v>0</v>
@@ -841,43 +858,43 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>V-33.444.555</v>
+        <v>V-34.666.777</v>
       </c>
       <c r="B11">
         <v>2000</v>
       </c>
       <c r="C11">
-        <v>300</v>
+        <v>200</v>
       </c>
       <c r="D11">
-        <v>227.43</v>
+        <v>100</v>
       </c>
       <c r="E11">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="F11">
-        <v>287.58</v>
+        <v>50</v>
       </c>
       <c r="G11">
-        <v>2.96</v>
+        <v>0</v>
       </c>
       <c r="H11">
-        <v>80</v>
+        <v>220</v>
       </c>
       <c r="I11">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="J11">
         <v>10</v>
       </c>
       <c r="K11">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="L11">
-        <v>45</v>
+        <v>80</v>
       </c>
       <c r="M11">
-        <v>174.61</v>
+        <v>0</v>
       </c>
       <c r="N11">
         <v>0</v>
@@ -885,51 +902,95 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>V-34.666.777</v>
+        <v>V-33.444.555</v>
       </c>
       <c r="B12">
-        <v>2900</v>
+        <v>2200</v>
       </c>
       <c r="C12">
-        <v>435</v>
+        <v>220</v>
       </c>
       <c r="D12">
-        <v>187.5</v>
+        <v>100</v>
       </c>
       <c r="E12">
-        <v>0</v>
+        <v>110</v>
       </c>
       <c r="F12">
-        <v>220.98</v>
+        <v>50</v>
       </c>
       <c r="G12">
-        <v>27.23</v>
+        <v>0</v>
       </c>
       <c r="H12">
-        <v>116</v>
+        <v>242</v>
       </c>
       <c r="I12">
-        <v>14.5</v>
+        <v>33</v>
       </c>
       <c r="J12">
-        <v>14.5</v>
+        <v>11</v>
       </c>
       <c r="K12">
-        <v>87</v>
+        <v>0</v>
       </c>
       <c r="L12">
-        <v>45</v>
+        <v>88</v>
       </c>
       <c r="M12">
-        <v>167.66</v>
+        <v>0</v>
       </c>
       <c r="N12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>V-35.111.223</v>
+      </c>
+      <c r="B13">
+        <v>2500</v>
+      </c>
+      <c r="C13">
+        <v>250</v>
+      </c>
+      <c r="D13">
+        <v>120</v>
+      </c>
+      <c r="E13">
+        <v>125</v>
+      </c>
+      <c r="F13">
+        <v>60</v>
+      </c>
+      <c r="G13">
+        <v>0</v>
+      </c>
+      <c r="H13">
+        <v>275</v>
+      </c>
+      <c r="I13">
+        <v>37.5</v>
+      </c>
+      <c r="J13">
+        <v>12.5</v>
+      </c>
+      <c r="K13">
+        <v>0</v>
+      </c>
+      <c r="L13">
+        <v>100</v>
+      </c>
+      <c r="M13">
+        <v>0</v>
+      </c>
+      <c r="N13">
         <v>0</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:N12"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:N13"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>